<commit_message>
Remove "Sponsors" it will be merged to "Fund Development > Sponsorships"
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrodua\Documents\new-file-management-system\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DE9FEB-B4D6-44A0-B802-5C04A9BEDBCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC01ACB-2995-42D2-A6CE-08001F11B93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="3645" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="96">
   <si>
     <t>FedYYC</t>
   </si>
@@ -263,9 +263,6 @@
     <t>Social Media</t>
   </si>
   <si>
-    <t>Sponsors</t>
-  </si>
-  <si>
     <t>Urban Planning Topics</t>
   </si>
   <si>
@@ -318,6 +315,15 @@
   </si>
   <si>
     <t>Manager Placemaking</t>
+  </si>
+  <si>
+    <t>Director Financial Literacy</t>
+  </si>
+  <si>
+    <t>Design Desk</t>
+  </si>
+  <si>
+    <t>Organization Culture &amp; EDIB</t>
   </si>
 </sst>
 </file>
@@ -607,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1066A4C7-BC62-4C6E-8946-8A1FB62B0DAC}">
-  <dimension ref="A1:Y72"/>
+  <dimension ref="A1:AA72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
@@ -618,25 +624,27 @@
     <col min="6" max="6" width="32.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.42578125" style="2" customWidth="1"/>
     <col min="8" max="8" width="19.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="33" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="29.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="18" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="27" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="51.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="21.140625" style="2" customWidth="1"/>
-    <col min="21" max="21" width="9.140625" style="2"/>
-    <col min="22" max="22" width="15.85546875" style="2" customWidth="1"/>
-    <col min="23" max="23" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="34" style="2" customWidth="1"/>
-    <col min="25" max="25" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="24.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="33" style="2" customWidth="1"/>
+    <col min="11" max="11" width="26" style="2" customWidth="1"/>
+    <col min="12" max="12" width="25.5703125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="29.28515625" style="2" customWidth="1"/>
+    <col min="15" max="16" width="18" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="27" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27" style="2" customWidth="1"/>
+    <col min="19" max="19" width="21.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="51.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="21.140625" style="2" customWidth="1"/>
+    <col min="23" max="23" width="9.140625" style="2"/>
+    <col min="24" max="24" width="15.85546875" style="2" customWidth="1"/>
+    <col min="25" max="25" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="34" style="2" customWidth="1"/>
+    <col min="27" max="27" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -650,10 +658,10 @@
         <v>4</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>5</v>
@@ -662,58 +670,64 @@
         <v>6</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="O1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -732,9 +746,6 @@
       <c r="H2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J2" s="2" t="s">
         <v>12</v>
       </c>
@@ -742,28 +753,28 @@
         <v>12</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>13</v>
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W2" s="2" t="s">
         <v>13</v>
@@ -771,8 +782,14 @@
       <c r="X2" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -785,16 +802,13 @@
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q3" s="2" t="s">
+      <c r="L3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R3" s="2" t="s">
@@ -806,8 +820,14 @@
       <c r="T3" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="U3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -823,9 +843,6 @@
       <c r="H4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J4" s="2" t="s">
         <v>12</v>
       </c>
@@ -838,14 +855,20 @@
       <c r="M4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="S4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -855,11 +878,14 @@
       <c r="D5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="K5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -869,11 +895,11 @@
       <c r="D6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="K6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -886,17 +912,17 @@
       <c r="H7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="L7" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>0</v>
       </c>
@@ -909,26 +935,29 @@
       <c r="E8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="L8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S8" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T8" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="U8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>0</v>
       </c>
@@ -938,14 +967,17 @@
       <c r="D9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="K9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -979,8 +1011,11 @@
       <c r="M10" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="N10" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -993,23 +1028,29 @@
       <c r="E11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M11" s="2" t="s">
+      <c r="K11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S11" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T11" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="U11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>0</v>
       </c>
@@ -1028,9 +1069,6 @@
       <c r="H12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J12" s="2" t="s">
         <v>12</v>
       </c>
@@ -1043,8 +1081,14 @@
       <c r="M12" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="N12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>0</v>
       </c>
@@ -1066,11 +1110,8 @@
       <c r="H13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="J13" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>13</v>
@@ -1079,22 +1120,25 @@
         <v>13</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="V13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="W13" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="X13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y13" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
@@ -1119,11 +1163,8 @@
       <c r="H14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J14" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>13</v>
@@ -1131,11 +1172,14 @@
       <c r="L14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Q14" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="M14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1145,8 +1189,29 @@
       <c r="D15" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="H15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>0</v>
       </c>
@@ -1159,9 +1224,6 @@
       <c r="H16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J16" s="2" t="s">
         <v>12</v>
       </c>
@@ -1177,7 +1239,7 @@
       <c r="N16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q16" s="2" t="s">
+      <c r="O16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R16" s="2" t="s">
@@ -1189,8 +1251,14 @@
       <c r="T16" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="U16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>0</v>
       </c>
@@ -1212,35 +1280,29 @@
       <c r="H17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I17" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="J17" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>13</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N17" s="2" t="s">
         <v>27</v>
       </c>
       <c r="S17" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="T17" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="U17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="V17" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="W17" s="2" t="s">
         <v>13</v>
@@ -1248,8 +1310,14 @@
       <c r="X17" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z17" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1271,32 +1339,26 @@
       <c r="H18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>13</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>13</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N18" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S18" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="T18" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="U18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="V18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W18" s="2" t="s">
         <v>13</v>
@@ -1304,8 +1366,14 @@
       <c r="X18" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z18" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>0</v>
       </c>
@@ -1330,35 +1398,29 @@
       <c r="H19" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I19" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="J19" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>13</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S19" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="T19" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="U19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="V19" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W19" s="2" t="s">
         <v>13</v>
@@ -1366,8 +1428,14 @@
       <c r="X19" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z19" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>0</v>
       </c>
@@ -1390,37 +1458,34 @@
         <v>12</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R20" s="2" t="s">
+      <c r="N20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S20" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="T20" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="U20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W20" s="2" t="s">
         <v>13</v>
@@ -1428,13 +1493,19 @@
       <c r="X20" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z20" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>27</v>
@@ -1451,9 +1522,6 @@
       <c r="H21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I21" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="J21" s="2" t="s">
         <v>27</v>
       </c>
@@ -1466,7 +1534,7 @@
       <c r="M21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="Q21" s="2" t="s">
+      <c r="N21" s="2" t="s">
         <v>27</v>
       </c>
       <c r="R21" s="2" t="s">
@@ -1479,10 +1547,10 @@
         <v>27</v>
       </c>
       <c r="U21" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="V21" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="W21" s="2" t="s">
         <v>13</v>
@@ -1490,13 +1558,19 @@
       <c r="X21" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z21" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>32</v>
@@ -1513,19 +1587,13 @@
       <c r="G22" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K22" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R22" s="2" t="s">
+      <c r="L22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S22" s="2" t="s">
@@ -1535,10 +1603,10 @@
         <v>12</v>
       </c>
       <c r="U22" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W22" s="2" t="s">
         <v>13</v>
@@ -1546,13 +1614,19 @@
       <c r="X22" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z22" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>23</v>
@@ -1572,9 +1646,6 @@
       <c r="H23" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I23" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J23" s="2" t="s">
         <v>12</v>
       </c>
@@ -1587,10 +1658,7 @@
       <c r="M23" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R23" s="2" t="s">
+      <c r="N23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S23" s="2" t="s">
@@ -1600,10 +1668,10 @@
         <v>12</v>
       </c>
       <c r="U23" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W23" s="2" t="s">
         <v>13</v>
@@ -1611,13 +1679,19 @@
       <c r="X23" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z23" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>35</v>
@@ -1637,9 +1711,6 @@
       <c r="H24" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I24" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J24" s="2" t="s">
         <v>12</v>
       </c>
@@ -1652,7 +1723,7 @@
       <c r="M24" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q24" s="2" t="s">
+      <c r="N24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R24" s="2" t="s">
@@ -1665,10 +1736,10 @@
         <v>12</v>
       </c>
       <c r="U24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W24" s="2" t="s">
         <v>13</v>
@@ -1676,13 +1747,19 @@
       <c r="X24" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z24" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>33</v>
@@ -1702,9 +1779,6 @@
       <c r="H25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J25" s="2" t="s">
         <v>12</v>
       </c>
@@ -1717,7 +1791,7 @@
       <c r="M25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q25" s="2" t="s">
+      <c r="N25" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R25" s="2" t="s">
@@ -1730,10 +1804,10 @@
         <v>12</v>
       </c>
       <c r="U25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W25" s="2" t="s">
         <v>13</v>
@@ -1741,13 +1815,19 @@
       <c r="X25" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z25" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>36</v>
@@ -1764,9 +1844,6 @@
       <c r="H26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I26" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J26" s="2" t="s">
         <v>12</v>
       </c>
@@ -1779,7 +1856,7 @@
       <c r="M26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q26" s="2" t="s">
+      <c r="N26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R26" s="2" t="s">
@@ -1792,10 +1869,10 @@
         <v>12</v>
       </c>
       <c r="U26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W26" s="2" t="s">
         <v>13</v>
@@ -1803,13 +1880,19 @@
       <c r="X26" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z26" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>37</v>
@@ -1823,16 +1906,13 @@
       <c r="F27" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J27" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K27" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q27" s="2" t="s">
+      <c r="L27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R27" s="2" t="s">
@@ -1845,10 +1925,10 @@
         <v>12</v>
       </c>
       <c r="U27" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V27" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W27" s="2" t="s">
         <v>13</v>
@@ -1856,13 +1936,19 @@
       <c r="X27" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z27" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>38</v>
@@ -1873,16 +1959,13 @@
       <c r="F28" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J28" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K28" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q28" s="2" t="s">
+      <c r="L28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R28" s="2" t="s">
@@ -1895,10 +1978,10 @@
         <v>12</v>
       </c>
       <c r="U28" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V28" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W28" s="2" t="s">
         <v>13</v>
@@ -1906,13 +1989,19 @@
       <c r="X28" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z28" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>39</v>
@@ -1929,19 +2018,13 @@
       <c r="G29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J29" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M29" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q29" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R29" s="2" t="s">
+      <c r="L29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N29" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S29" s="2" t="s">
@@ -1951,10 +2034,10 @@
         <v>12</v>
       </c>
       <c r="U29" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V29" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W29" s="2" t="s">
         <v>13</v>
@@ -1962,8 +2045,14 @@
       <c r="X29" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z29" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>0</v>
       </c>
@@ -1979,9 +2068,6 @@
       <c r="H30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I30" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J30" s="2" t="s">
         <v>12</v>
       </c>
@@ -1994,8 +2080,14 @@
       <c r="M30" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="N30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R30" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>0</v>
       </c>
@@ -2011,26 +2103,26 @@
       <c r="G31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y31" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="K31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA31" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>0</v>
       </c>
@@ -2046,17 +2138,17 @@
       <c r="G32" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R32" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="K32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T32" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>0</v>
       </c>
@@ -2072,14 +2164,14 @@
       <c r="E33" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J33" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R33" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="K33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T33" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>0</v>
       </c>
@@ -2092,11 +2184,11 @@
       <c r="D34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="X34" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Z34" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>0</v>
       </c>
@@ -2109,11 +2201,11 @@
       <c r="D35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Y35" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AA35" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>0</v>
       </c>
@@ -2121,22 +2213,23 @@
         <v>41</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>46</v>
+        <v>95</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R36" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="H36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA36" s="2"/>
+    </row>
+    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>0</v>
       </c>
@@ -2144,16 +2237,22 @@
         <v>41</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L37" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="E37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T37" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>0</v>
       </c>
@@ -2161,101 +2260,107 @@
         <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="D39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W39" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D40" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y40" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>0</v>
       </c>
@@ -2263,70 +2368,16 @@
         <v>2</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F41" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O41" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W41" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>0</v>
       </c>
@@ -2334,25 +2385,76 @@
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E42" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="F42" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="N42" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="O42" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="P42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y42" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>0</v>
       </c>
@@ -2360,7 +2462,7 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>12</v>
@@ -2368,14 +2470,17 @@
       <c r="F43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N43" s="2" t="s">
+      <c r="G43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O43" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="P43" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>0</v>
       </c>
@@ -2383,7 +2488,7 @@
         <v>2</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>12</v>
@@ -2394,8 +2499,11 @@
       <c r="O44" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="P44" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>0</v>
       </c>
@@ -2403,7 +2511,7 @@
         <v>2</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>12</v>
@@ -2411,20 +2519,14 @@
       <c r="F45" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G45" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K45" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N45" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="O45" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="P45" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -2432,245 +2534,239 @@
         <v>2</v>
       </c>
       <c r="C46" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P46" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O46" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B47" s="1" t="s">
+      <c r="D47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P47" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T47" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B48" s="1" t="s">
+      <c r="D48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V48" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W48" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B49" s="1" t="s">
+      <c r="D49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y49" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M49" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="D50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="R50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W50" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C51" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q51" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T51" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="U51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y51" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>0</v>
       </c>
@@ -2678,7 +2774,7 @@
         <v>58</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>12</v>
@@ -2707,10 +2803,7 @@
       <c r="M52" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q52" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R52" s="2" t="s">
+      <c r="N52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S52" s="2" t="s">
@@ -2725,11 +2818,8 @@
       <c r="V52" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="W52" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>0</v>
       </c>
@@ -2737,310 +2827,376 @@
         <v>58</v>
       </c>
       <c r="C53" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y53" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T53" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B54" s="1" t="s">
+      <c r="D54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V54" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="55" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T54" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B55" s="1" t="s">
+      <c r="D55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V55" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W55" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B56" s="1" t="s">
+      <c r="D56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y56" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="57" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T56" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B57" s="1" t="s">
+      <c r="D57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V57" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="58" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S57" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="D58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="R58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W58" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C59" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="R59" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="S59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y59" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="60" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
@@ -3048,7 +3204,7 @@
         <v>65</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>12</v>
@@ -3056,38 +3212,14 @@
       <c r="G60" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K60" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S60" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T60" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>0</v>
       </c>
@@ -3095,23 +3227,17 @@
         <v>65</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G61" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J61" s="2" t="s">
         <v>12</v>
       </c>
@@ -3124,7 +3250,7 @@
       <c r="M61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q61" s="2" t="s">
+      <c r="N61" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R61" s="2" t="s">
@@ -3139,8 +3265,11 @@
       <c r="U61" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V61" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>0</v>
       </c>
@@ -3148,7 +3277,7 @@
         <v>65</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>12</v>
@@ -3156,9 +3285,6 @@
       <c r="E62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3183,15 +3309,6 @@
       <c r="N62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3211,7 +3328,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>0</v>
       </c>
@@ -3219,11 +3336,17 @@
         <v>65</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3245,6 +3368,15 @@
       <c r="M63" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="N63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="Q63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3257,8 +3389,23 @@
       <c r="T63" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="U63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y63" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="64" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>0</v>
       </c>
@@ -3266,7 +3413,7 @@
         <v>65</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>12</v>
@@ -3277,9 +3424,6 @@
       <c r="H64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I64" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3292,7 +3436,7 @@
       <c r="M64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q64" s="2" t="s">
+      <c r="N64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R64" s="2" t="s">
@@ -3304,8 +3448,14 @@
       <c r="T64" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="U64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V64" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="65" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>0</v>
       </c>
@@ -3313,211 +3463,244 @@
         <v>65</v>
       </c>
       <c r="C65" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V65" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="66" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L65" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B66" s="1" t="s">
+      <c r="D66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R66" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="67" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q66" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B67" s="1" t="s">
+      <c r="D67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S67" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="68" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B68" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L67" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A68" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="1" t="s">
+      <c r="D68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R68" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="69" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T68" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B69" s="1" t="s">
+      <c r="D69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V69" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="70" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T69" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B70" s="1" t="s">
+      <c r="D70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R70" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B71" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M70" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B71" s="1" t="s">
+      <c r="D71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T71" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="72" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B72" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R71" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="D72" s="2" t="s">
         <v>12</v>
       </c>
@@ -3542,7 +3725,7 @@
       <c r="M72" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q72" s="2" t="s">
+      <c r="N72" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R72" s="2" t="s">
@@ -3561,6 +3744,12 @@
         <v>12</v>
       </c>
       <c r="W72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y72" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3570,7 +3759,7 @@
       <formula>NOT(ISBLANK($C2))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:Y1048576">
+  <conditionalFormatting sqref="D1:AA1048576">
     <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>"RW"</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: update generated permission and AD derivatives
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrodua\Documents\new-file-management-system\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Documents\new-file-management-system\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC01ACB-2995-42D2-A6CE-08001F11B93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD0AA03-BE19-4FD4-B866-48B899CE9C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
+    <workbookView xWindow="57480" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="97">
   <si>
     <t>FedYYC</t>
   </si>
@@ -324,6 +324,9 @@
   </si>
   <si>
     <t>Organization Culture &amp; EDIB</t>
+  </si>
+  <si>
+    <t>Test Committee</t>
   </si>
 </sst>
 </file>
@@ -613,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1066A4C7-BC62-4C6E-8946-8A1FB62B0DAC}">
-  <dimension ref="A1:AA72"/>
+  <dimension ref="A1:AA73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
@@ -1184,31 +1187,40 @@
         <v>0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="H15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V15" s="2" t="s">
-        <v>12</v>
+      <c r="K15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
@@ -1216,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>12</v>
@@ -1224,31 +1236,16 @@
       <c r="H16" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I16" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O16" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="U16" s="2" t="s">
@@ -1263,58 +1260,46 @@
         <v>0</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="V17" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
@@ -1324,17 +1309,17 @@
       <c r="B18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>13</v>
@@ -1342,6 +1327,9 @@
       <c r="J18" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="K18" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="L18" s="2" t="s">
         <v>13</v>
       </c>
@@ -1349,16 +1337,16 @@
         <v>13</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W18" s="2" t="s">
         <v>13</v>
@@ -1381,14 +1369,11 @@
         <v>31</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F19" s="2" t="s">
         <v>13</v>
       </c>
@@ -1400,9 +1385,6 @@
       </c>
       <c r="J19" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>13</v>
@@ -1443,7 +1425,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>12</v>
@@ -1458,19 +1440,19 @@
         <v>12</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N20" s="2" t="s">
         <v>12</v>
@@ -1482,9 +1464,6 @@
         <v>12</v>
       </c>
       <c r="U20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="W20" s="2" t="s">
@@ -1505,52 +1484,52 @@
         <v>0</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>91</v>
+        <v>31</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W21" s="2" t="s">
         <v>13</v>
@@ -1572,14 +1551,11 @@
       <c r="B22" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>13</v>
@@ -1587,26 +1563,38 @@
       <c r="G22" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="H22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="K22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W22" s="2" t="s">
         <v>13</v>
@@ -1629,7 +1617,7 @@
         <v>91</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>12</v>
@@ -1641,21 +1629,12 @@
         <v>13</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N23" s="2" t="s">
@@ -1694,7 +1673,7 @@
         <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>12</v>
@@ -1724,9 +1703,6 @@
         <v>12</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S24" s="2" t="s">
@@ -1762,7 +1738,7 @@
         <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>12</v>
@@ -1830,9 +1806,12 @@
         <v>91</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F26" s="2" t="s">
@@ -1895,21 +1874,30 @@
         <v>91</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F27" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N27" s="2" t="s">
@@ -1951,9 +1939,12 @@
         <v>91</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F28" s="2" t="s">
@@ -2004,20 +1995,14 @@
         <v>91</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K29" s="2" t="s">
         <v>12</v>
       </c>
@@ -2025,6 +2010,9 @@
         <v>12</v>
       </c>
       <c r="N29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R29" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S29" s="2" t="s">
@@ -2057,34 +2045,55 @@
         <v>0</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>40</v>
+        <v>91</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="G30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K30" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M30" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R30" s="2" t="s">
-        <v>12</v>
+      <c r="S30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="X30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z30" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
@@ -2092,34 +2101,34 @@
         <v>0</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R31" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
@@ -2129,23 +2138,32 @@
       <c r="B32" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="D32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="Z32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA32" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
@@ -2156,15 +2174,18 @@
         <v>41</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S33" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T33" s="2" t="s">
@@ -2179,12 +2200,18 @@
         <v>41</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Z34" s="2" t="s">
+      <c r="E34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T34" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2196,12 +2223,12 @@
         <v>41</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="AA35" s="2" t="s">
+      <c r="Z35" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2213,21 +2240,14 @@
         <v>41</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA36" s="2"/>
+      <c r="AA36" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
@@ -2237,20 +2257,21 @@
         <v>41</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>46</v>
+        <v>95</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T37" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="H37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA37" s="2"/>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
@@ -2260,12 +2281,18 @@
         <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M38" s="2" t="s">
+      <c r="E38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T38" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2277,12 +2304,12 @@
         <v>41</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H39" s="2" t="s">
+      <c r="M39" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2291,73 +2318,16 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>2</v>
+        <v>41</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y40" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.25">
@@ -2367,14 +2337,71 @@
       <c r="B41" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D41" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y41" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
@@ -2385,73 +2412,13 @@
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F42" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O42" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P42" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y42" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
@@ -2462,22 +2429,73 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E43" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="F43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="O43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="P43" s="2" t="s">
         <v>12</v>
+      </c>
+      <c r="Q43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y43" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.25">
@@ -2488,12 +2506,15 @@
         <v>2</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O44" s="2" t="s">
@@ -2511,7 +2532,7 @@
         <v>2</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>12</v>
@@ -2534,18 +2555,12 @@
         <v>2</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O46" s="2" t="s">
@@ -2563,7 +2578,7 @@
         <v>2</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>12</v>
@@ -2589,30 +2604,27 @@
         <v>0</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>55</v>
+        <v>2</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V48" s="2" t="s">
+      <c r="F48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P48" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2621,32 +2633,14 @@
         <v>0</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K49" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M49" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N49" s="2" t="s">
         <v>12</v>
       </c>
@@ -2663,15 +2657,6 @@
         <v>12</v>
       </c>
       <c r="V49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y49" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2680,14 +2665,20 @@
         <v>0</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G50" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H50" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I50" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J50" s="2" t="s">
         <v>12</v>
       </c>
@@ -2704,6 +2695,27 @@
         <v>12</v>
       </c>
       <c r="R50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y50" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2712,58 +2724,31 @@
         <v>0</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="R51" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
@@ -2773,50 +2758,56 @@
       <c r="B52" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C52" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="W52" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X52" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y52" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
@@ -2827,7 +2818,7 @@
         <v>58</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>12</v>
@@ -2869,15 +2860,6 @@
         <v>12</v>
       </c>
       <c r="V53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y53" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2889,7 +2871,7 @@
         <v>58</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>12</v>
@@ -2931,6 +2913,15 @@
         <v>12</v>
       </c>
       <c r="V54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y54" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2939,11 +2930,20 @@
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H55" s="2" t="s">
         <v>12</v>
       </c>
@@ -2963,9 +2963,6 @@
         <v>12</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R55" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S55" s="2" t="s">
@@ -2986,20 +2983,11 @@
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H56" s="2" t="s">
         <v>12</v>
       </c>
@@ -3034,15 +3022,6 @@
         <v>12</v>
       </c>
       <c r="V56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y56" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3051,17 +3030,26 @@
         <v>0</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G57" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J57" s="2" t="s">
         <v>12</v>
       </c>
@@ -3090,6 +3078,15 @@
         <v>12</v>
       </c>
       <c r="V57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y57" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3098,11 +3095,14 @@
         <v>0</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G58" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H58" s="2" t="s">
         <v>12</v>
       </c>
@@ -3115,10 +3115,25 @@
       <c r="L58" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R58" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="S58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T58" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="U58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V58" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3127,73 +3142,28 @@
         <v>0</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="R59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
@@ -3203,20 +3173,71 @@
       <c r="B60" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C60" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S60" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="T60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="U60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y60" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
@@ -3227,7 +3248,7 @@
         <v>65</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>12</v>
@@ -3235,37 +3256,10 @@
       <c r="G61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V61" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3277,23 +3271,17 @@
         <v>65</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3322,9 +3310,6 @@
         <v>12</v>
       </c>
       <c r="V62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W62" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3336,7 +3321,7 @@
         <v>65</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>12</v>
@@ -3344,9 +3329,6 @@
       <c r="E63" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F63" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3371,15 +3353,6 @@
       <c r="N63" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q63" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3396,12 +3369,6 @@
         <v>12</v>
       </c>
       <c r="W63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y63" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3413,17 +3380,26 @@
         <v>65</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I64" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3439,6 +3415,15 @@
       <c r="N64" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q64" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3452,6 +3437,15 @@
         <v>12</v>
       </c>
       <c r="V64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y64" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3463,7 +3457,7 @@
         <v>65</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>12</v>
@@ -3513,18 +3507,45 @@
         <v>65</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K66" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M66" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="N66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V66" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3533,36 +3554,21 @@
         <v>0</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L67" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S67" s="2" t="s">
+      <c r="R67" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3571,12 +3577,21 @@
         <v>0</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G68" s="2" t="s">
+      <c r="F68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J68" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K68" s="2" t="s">
@@ -3588,7 +3603,10 @@
       <c r="M68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R68" s="2" t="s">
+      <c r="N68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S68" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3597,7 +3615,7 @@
         <v>0</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>12</v>
@@ -3605,15 +3623,6 @@
       <c r="G69" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J69" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K69" s="2" t="s">
         <v>12</v>
       </c>
@@ -3623,22 +3632,7 @@
       <c r="M69" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N69" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V69" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3647,11 +3641,29 @@
         <v>0</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L70" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M70" s="2" t="s">
         <v>12</v>
       </c>
@@ -3659,6 +3671,18 @@
         <v>12</v>
       </c>
       <c r="R70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V70" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3667,20 +3691,11 @@
         <v>0</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K71" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M71" s="2" t="s">
         <v>12</v>
       </c>
@@ -3688,9 +3703,6 @@
         <v>12</v>
       </c>
       <c r="R71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T71" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3699,62 +3711,94 @@
         <v>0</v>
       </c>
       <c r="B72" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T72" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="73" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B73" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y72" s="2" t="s">
+      <c r="D73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y73" s="2" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B1000">
+  <conditionalFormatting sqref="A2:B1001">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(ISBLANK($C2))</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: updated derivatives csv
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Documents\new-file-management-system\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD0AA03-BE19-4FD4-B866-48B899CE9C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31AF39A-6F2A-4AEF-8DA4-300B78270E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="95">
   <si>
     <t>FedYYC</t>
   </si>
@@ -321,12 +321,6 @@
   </si>
   <si>
     <t>Design Desk</t>
-  </si>
-  <si>
-    <t>Organization Culture &amp; EDIB</t>
-  </si>
-  <si>
-    <t>Test Committee</t>
   </si>
 </sst>
 </file>
@@ -616,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1066A4C7-BC62-4C6E-8946-8A1FB62B0DAC}">
-  <dimension ref="A1:AA73"/>
+  <dimension ref="A1:AA71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
@@ -901,6 +895,9 @@
       <c r="K6" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="S6" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -1187,40 +1184,31 @@
         <v>0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>96</v>
+        <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="H15" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I15" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="S15" s="2" t="s">
-        <v>13</v>
+      <c r="N15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
@@ -1228,7 +1216,7 @@
         <v>0</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>12</v>
@@ -1236,16 +1224,31 @@
       <c r="H16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J16" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="K16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N16" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O16" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="U16" s="2" t="s">
@@ -1260,46 +1263,58 @@
         <v>0</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="W17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="X17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z17" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
@@ -1309,17 +1324,17 @@
       <c r="B18" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="C18" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="D18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>13</v>
@@ -1327,9 +1342,6 @@
       <c r="J18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="L18" s="2" t="s">
         <v>13</v>
       </c>
@@ -1337,16 +1349,16 @@
         <v>13</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W18" s="2" t="s">
         <v>13</v>
@@ -1369,11 +1381,14 @@
         <v>31</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E19" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="F19" s="2" t="s">
         <v>13</v>
       </c>
@@ -1385,6 +1400,9 @@
       </c>
       <c r="J19" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>13</v>
@@ -1425,7 +1443,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>12</v>
@@ -1440,19 +1458,19 @@
         <v>12</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N20" s="2" t="s">
         <v>12</v>
@@ -1464,6 +1482,9 @@
         <v>12</v>
       </c>
       <c r="U20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="W20" s="2" t="s">
@@ -1484,52 +1505,52 @@
         <v>0</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="R21" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V21" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W21" s="2" t="s">
         <v>13</v>
@@ -1551,11 +1572,14 @@
       <c r="B22" s="1" t="s">
         <v>91</v>
       </c>
+      <c r="C22" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="D22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>13</v>
@@ -1563,38 +1587,26 @@
       <c r="G22" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="K22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W22" s="2" t="s">
         <v>13</v>
@@ -1617,7 +1629,7 @@
         <v>91</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>12</v>
@@ -1629,12 +1641,21 @@
         <v>13</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N23" s="2" t="s">
@@ -1673,7 +1694,7 @@
         <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>12</v>
@@ -1703,6 +1724,9 @@
         <v>12</v>
       </c>
       <c r="N24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S24" s="2" t="s">
@@ -1738,7 +1762,7 @@
         <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>12</v>
@@ -1806,12 +1830,9 @@
         <v>91</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F26" s="2" t="s">
@@ -1874,30 +1895,21 @@
         <v>91</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E27" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="F27" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N27" s="2" t="s">
@@ -1939,12 +1951,9 @@
         <v>91</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F28" s="2" t="s">
@@ -1995,14 +2004,20 @@
         <v>91</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E29" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="F29" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G29" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K29" s="2" t="s">
         <v>12</v>
       </c>
@@ -2010,9 +2025,6 @@
         <v>12</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R29" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S29" s="2" t="s">
@@ -2045,55 +2057,34 @@
         <v>0</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="G30" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K30" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M30" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z30" s="2" t="s">
-        <v>13</v>
+      <c r="R30" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
@@ -2101,34 +2092,34 @@
         <v>0</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="S31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA31" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
@@ -2138,32 +2129,23 @@
       <c r="B32" s="1" t="s">
         <v>41</v>
       </c>
+      <c r="C32" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="D32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
@@ -2174,18 +2156,15 @@
         <v>41</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="E33" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S33" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T33" s="2" t="s">
@@ -2200,18 +2179,12 @@
         <v>41</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T34" s="2" t="s">
+      <c r="Z34" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2223,12 +2196,12 @@
         <v>41</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Z35" s="2" t="s">
+      <c r="AA35" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2240,12 +2213,18 @@
         <v>41</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="AA36" s="2" t="s">
+      <c r="E36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T36" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2257,21 +2236,14 @@
         <v>41</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>95</v>
+        <v>47</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AA37" s="2"/>
+      <c r="M37" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
@@ -2281,18 +2253,12 @@
         <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T38" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2301,16 +2267,73 @@
         <v>0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X39" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y39" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
@@ -2318,15 +2341,15 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H40" s="2" t="s">
+      <c r="F40" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2337,17 +2360,20 @@
       <c r="B41" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C41" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="D41" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>27</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>27</v>
@@ -2371,10 +2397,10 @@
         <v>27</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="P41" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="Q41" s="2" t="s">
         <v>27</v>
@@ -2412,12 +2438,21 @@
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P42" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2429,73 +2464,19 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E43" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G43" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N43" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="O43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="P43" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="Q43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y43" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.25">
@@ -2506,15 +2487,12 @@
         <v>2</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O44" s="2" t="s">
@@ -2532,12 +2510,18 @@
         <v>2</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O45" s="2" t="s">
@@ -2555,12 +2539,18 @@
         <v>2</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O46" s="2" t="s">
@@ -2575,27 +2565,30 @@
         <v>0</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P47" s="2" t="s">
+      <c r="K47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V47" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2604,27 +2597,57 @@
         <v>0</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F48" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G48" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="L48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P48" s="2" t="s">
+      <c r="M48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y48" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2633,30 +2656,30 @@
         <v>0</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K49" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N49" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V49" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2665,58 +2688,58 @@
         <v>0</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="X50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="Y50" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
@@ -2724,14 +2747,26 @@
         <v>0</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H51" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I51" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J51" s="2" t="s">
         <v>12</v>
       </c>
@@ -2747,7 +2782,16 @@
       <c r="N51" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R51" s="2" t="s">
+      <c r="S51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V51" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2758,56 +2802,59 @@
       <c r="B52" s="1" t="s">
         <v>58</v>
       </c>
+      <c r="C52" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="D52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="X52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="Y52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
@@ -2818,7 +2865,7 @@
         <v>58</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>12</v>
@@ -2868,20 +2915,11 @@
         <v>0</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H54" s="2" t="s">
         <v>12</v>
       </c>
@@ -2903,6 +2941,9 @@
       <c r="N54" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="R54" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="S54" s="2" t="s">
         <v>12</v>
       </c>
@@ -2913,15 +2954,6 @@
         <v>12</v>
       </c>
       <c r="V54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y54" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2930,10 +2962,7 @@
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>12</v>
@@ -2941,6 +2970,9 @@
       <c r="E55" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="F55" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G55" s="2" t="s">
         <v>12</v>
       </c>
@@ -2965,6 +2997,9 @@
       <c r="N55" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="R55" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="S55" s="2" t="s">
         <v>12</v>
       </c>
@@ -2975,6 +3010,15 @@
         <v>12</v>
       </c>
       <c r="V55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y55" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2983,15 +3027,15 @@
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G56" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I56" s="2" t="s">
         <v>12</v>
       </c>
       <c r="J56" s="2" t="s">
@@ -3030,26 +3074,14 @@
         <v>0</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I57" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J57" s="2" t="s">
         <v>12</v>
       </c>
@@ -3059,34 +3091,10 @@
       <c r="L57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N57" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T57" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="U57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y57" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3095,46 +3103,73 @@
         <v>0</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="O58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q58" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="R58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V58" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="W58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y58" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.25">
@@ -3142,27 +3177,21 @@
         <v>0</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H59" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J59" s="2" t="s">
+      <c r="G59" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L59" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R59" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U59" s="2" t="s">
+      <c r="T59" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3173,71 +3202,47 @@
       <c r="B60" s="1" t="s">
         <v>65</v>
       </c>
+      <c r="C60" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="D60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="R60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
@@ -3248,18 +3253,54 @@
         <v>65</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E61" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G61" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K61" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S61" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="T61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W61" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3271,17 +3312,26 @@
         <v>65</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I62" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3297,6 +3347,15 @@
       <c r="N62" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q62" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3310,6 +3369,15 @@
         <v>12</v>
       </c>
       <c r="V62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y62" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3321,23 +3389,17 @@
         <v>65</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E63" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G63" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I63" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3366,9 +3428,6 @@
         <v>12</v>
       </c>
       <c r="V63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W63" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3380,26 +3439,17 @@
         <v>65</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I64" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3415,15 +3465,6 @@
       <c r="N64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q64" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3437,15 +3478,6 @@
         <v>12</v>
       </c>
       <c r="V64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y64" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3457,45 +3489,18 @@
         <v>65</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J65" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K65" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L65" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M65" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N65" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V65" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3504,20 +3509,20 @@
         <v>0</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J66" s="2" t="s">
         <v>12</v>
       </c>
@@ -3533,19 +3538,7 @@
       <c r="N66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R66" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="S66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V66" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3554,15 +3547,18 @@
         <v>0</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G67" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L67" s="2" t="s">
         <v>12</v>
       </c>
       <c r="M67" s="2" t="s">
@@ -3577,12 +3573,12 @@
         <v>0</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F68" s="2" t="s">
+      <c r="G68" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H68" s="2" t="s">
@@ -3606,7 +3602,19 @@
       <c r="N68" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="R68" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="S68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V68" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3615,21 +3623,15 @@
         <v>0</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L69" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N69" s="2" t="s">
         <v>12</v>
       </c>
       <c r="R69" s="2" t="s">
@@ -3641,29 +3643,20 @@
         <v>0</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="F70" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J70" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L70" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M70" s="2" t="s">
         <v>12</v>
       </c>
@@ -3673,16 +3666,7 @@
       <c r="R70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S70" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V70" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3691,11 +3675,29 @@
         <v>0</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L71" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M71" s="2" t="s">
         <v>12</v>
       </c>
@@ -3705,100 +3707,30 @@
       <c r="R71" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="72" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T72" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="73" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y73" s="2" t="s">
+      <c r="S71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y71" s="2" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B1001">
+  <conditionalFormatting sqref="A2:B999">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(ISBLANK($C2))</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: update generated CSV files
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Documents\new-file-management-system\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31AF39A-6F2A-4AEF-8DA4-300B78270E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B18E75A-F698-49F5-B988-FF004E04510E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="95">
   <si>
     <t>FedYYC</t>
   </si>
@@ -895,9 +895,6 @@
       <c r="K6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">

</xml_diff>

<commit_message>
docs: update generated CSV
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Documents\new-file-management-system\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B18E75A-F698-49F5-B988-FF004E04510E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AA3854F-7917-400E-9A6E-A8DF0F1B941E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="95">
   <si>
     <t>FedYYC</t>
   </si>
@@ -2570,6 +2570,9 @@
       <c r="K47" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L47" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N47" s="2" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
docs: update generated CSVs
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0293660-BBD6-48F4-A671-FD29E78B3BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F4B782-8817-4710-9DF4-CF1DC769A440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="97">
   <si>
     <t>FedYYC</t>
   </si>
@@ -321,6 +321,12 @@
   </si>
   <si>
     <t>Design Desk</t>
+  </si>
+  <si>
+    <t>PIP</t>
+  </si>
+  <si>
+    <t>NewFolder</t>
   </si>
 </sst>
 </file>
@@ -610,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1066A4C7-BC62-4C6E-8946-8A1FB62B0DAC}">
-  <dimension ref="A1:AA71"/>
+  <dimension ref="A1:AA73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
@@ -1181,31 +1187,40 @@
         <v>0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="H15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V15" s="2" t="s">
-        <v>12</v>
+      <c r="K15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
@@ -1213,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>12</v>
@@ -1221,31 +1236,16 @@
       <c r="H16" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I16" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O16" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="U16" s="2" t="s">
@@ -1260,58 +1260,46 @@
         <v>0</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="V17" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
@@ -1321,17 +1309,17 @@
       <c r="B18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>13</v>
@@ -1339,6 +1327,9 @@
       <c r="J18" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="K18" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="L18" s="2" t="s">
         <v>13</v>
       </c>
@@ -1346,16 +1337,16 @@
         <v>13</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W18" s="2" t="s">
         <v>13</v>
@@ -1378,14 +1369,11 @@
         <v>31</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F19" s="2" t="s">
         <v>13</v>
       </c>
@@ -1397,9 +1385,6 @@
       </c>
       <c r="J19" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>13</v>
@@ -1440,7 +1425,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>12</v>
@@ -1455,19 +1440,19 @@
         <v>12</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N20" s="2" t="s">
         <v>12</v>
@@ -1479,9 +1464,6 @@
         <v>12</v>
       </c>
       <c r="U20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="W20" s="2" t="s">
@@ -1502,52 +1484,52 @@
         <v>0</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>91</v>
+        <v>31</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V21" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W21" s="2" t="s">
         <v>13</v>
@@ -1569,14 +1551,11 @@
       <c r="B22" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>13</v>
@@ -1584,26 +1563,38 @@
       <c r="G22" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="H22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="K22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W22" s="2" t="s">
         <v>13</v>
@@ -1626,7 +1617,7 @@
         <v>91</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>12</v>
@@ -1638,21 +1629,12 @@
         <v>13</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N23" s="2" t="s">
@@ -1691,7 +1673,7 @@
         <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>12</v>
@@ -1721,9 +1703,6 @@
         <v>12</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S24" s="2" t="s">
@@ -1759,7 +1738,7 @@
         <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>12</v>
@@ -1827,9 +1806,12 @@
         <v>91</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F26" s="2" t="s">
@@ -1892,21 +1874,30 @@
         <v>91</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F27" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N27" s="2" t="s">
@@ -1948,9 +1939,12 @@
         <v>91</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F28" s="2" t="s">
@@ -2001,20 +1995,14 @@
         <v>91</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K29" s="2" t="s">
         <v>12</v>
       </c>
@@ -2022,6 +2010,9 @@
         <v>12</v>
       </c>
       <c r="N29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R29" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S29" s="2" t="s">
@@ -2054,34 +2045,55 @@
         <v>0</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>40</v>
+        <v>91</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="G30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K30" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M30" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R30" s="2" t="s">
-        <v>12</v>
+      <c r="S30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="X30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z30" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
@@ -2089,34 +2101,34 @@
         <v>0</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z31" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA31" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R31" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
@@ -2126,23 +2138,32 @@
       <c r="B32" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="D32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="Z32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA32" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
@@ -2153,15 +2174,18 @@
         <v>41</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S33" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T33" s="2" t="s">
@@ -2176,12 +2200,18 @@
         <v>41</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Z34" s="2" t="s">
+      <c r="E34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T34" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2193,12 +2223,12 @@
         <v>41</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="AA35" s="2" t="s">
+      <c r="Z35" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2210,18 +2240,12 @@
         <v>41</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T36" s="2" t="s">
+      <c r="AA36" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2233,12 +2257,18 @@
         <v>41</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M37" s="2" t="s">
+      <c r="E37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T37" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2250,12 +2280,12 @@
         <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="M38" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2264,73 +2294,16 @@
         <v>0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>2</v>
+        <v>41</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X39" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y39" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
@@ -2340,14 +2313,71 @@
       <c r="B40" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D40" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y40" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.25">
@@ -2358,73 +2388,13 @@
         <v>2</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F41" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O41" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P41" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y41" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
@@ -2435,22 +2405,73 @@
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E42" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="F42" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="O42" s="2" t="s">
         <v>12</v>
       </c>
       <c r="P42" s="2" t="s">
         <v>12</v>
+      </c>
+      <c r="Q42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y42" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
@@ -2461,12 +2482,15 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O43" s="2" t="s">
@@ -2484,7 +2508,7 @@
         <v>2</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>12</v>
@@ -2507,18 +2531,12 @@
         <v>2</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O45" s="2" t="s">
@@ -2536,7 +2554,7 @@
         <v>2</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>12</v>
@@ -2562,33 +2580,27 @@
         <v>0</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>55</v>
+        <v>2</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K47" s="2" t="s">
+      <c r="F47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U47" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V47" s="2" t="s">
+      <c r="O47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P47" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2597,32 +2609,17 @@
         <v>0</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K48" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M48" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N48" s="2" t="s">
         <v>12</v>
       </c>
@@ -2639,15 +2636,6 @@
         <v>12</v>
       </c>
       <c r="V48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y48" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2656,14 +2644,20 @@
         <v>0</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H49" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J49" s="2" t="s">
         <v>12</v>
       </c>
@@ -2680,6 +2674,27 @@
         <v>12</v>
       </c>
       <c r="R49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y49" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2688,58 +2703,31 @@
         <v>0</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y50" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="R50" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
@@ -2749,50 +2737,56 @@
       <c r="B51" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C51" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="W51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y51" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
@@ -2803,7 +2797,7 @@
         <v>58</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>12</v>
@@ -2845,15 +2839,6 @@
         <v>12</v>
       </c>
       <c r="V52" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W52" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X52" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y52" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2865,7 +2850,7 @@
         <v>58</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>12</v>
@@ -2907,6 +2892,15 @@
         <v>12</v>
       </c>
       <c r="V53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y53" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2915,11 +2909,20 @@
         <v>0</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H54" s="2" t="s">
         <v>12</v>
       </c>
@@ -2939,9 +2942,6 @@
         <v>12</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R54" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S54" s="2" t="s">
@@ -2962,20 +2962,11 @@
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H55" s="2" t="s">
         <v>12</v>
       </c>
@@ -3010,15 +3001,6 @@
         <v>12</v>
       </c>
       <c r="V55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y55" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3027,17 +3009,26 @@
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G56" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I56" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J56" s="2" t="s">
         <v>12</v>
       </c>
@@ -3066,6 +3057,15 @@
         <v>12</v>
       </c>
       <c r="V56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y56" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3074,11 +3074,14 @@
         <v>0</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H57" s="2" t="s">
         <v>12</v>
       </c>
@@ -3091,10 +3094,25 @@
       <c r="L57" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R57" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="S57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="U57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V57" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3103,73 +3121,28 @@
         <v>0</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="R58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y58" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.25">
@@ -3179,20 +3152,71 @@
       <c r="B59" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C59" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="L59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="T59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="U59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y59" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
@@ -3203,7 +3227,7 @@
         <v>65</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>12</v>
@@ -3211,37 +3235,10 @@
       <c r="G60" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K60" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S60" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V60" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3253,23 +3250,17 @@
         <v>65</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G61" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J61" s="2" t="s">
         <v>12</v>
       </c>
@@ -3298,9 +3289,6 @@
         <v>12</v>
       </c>
       <c r="V61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W61" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3312,7 +3300,7 @@
         <v>65</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>12</v>
@@ -3320,9 +3308,6 @@
       <c r="E62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3347,15 +3332,6 @@
       <c r="N62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3372,12 +3348,6 @@
         <v>12</v>
       </c>
       <c r="W62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y62" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3389,17 +3359,26 @@
         <v>65</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G63" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3415,6 +3394,15 @@
       <c r="N63" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3428,6 +3416,15 @@
         <v>12</v>
       </c>
       <c r="V63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y63" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3439,7 +3436,7 @@
         <v>65</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>12</v>
@@ -3489,18 +3486,45 @@
         <v>65</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K65" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L65" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M65" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="N65" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V65" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3509,36 +3533,21 @@
         <v>0</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J66" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L66" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S66" s="2" t="s">
+      <c r="R66" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3547,12 +3556,21 @@
         <v>0</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G67" s="2" t="s">
+      <c r="F67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J67" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K67" s="2" t="s">
@@ -3564,7 +3582,10 @@
       <c r="M67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R67" s="2" t="s">
+      <c r="N67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S67" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3573,7 +3594,7 @@
         <v>0</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>12</v>
@@ -3581,15 +3602,6 @@
       <c r="G68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J68" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K68" s="2" t="s">
         <v>12</v>
       </c>
@@ -3599,22 +3611,7 @@
       <c r="M68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N68" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V68" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3623,11 +3620,29 @@
         <v>0</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M69" s="2" t="s">
         <v>12</v>
       </c>
@@ -3635,6 +3650,18 @@
         <v>12</v>
       </c>
       <c r="R69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V69" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3643,20 +3670,11 @@
         <v>0</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K70" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M70" s="2" t="s">
         <v>12</v>
       </c>
@@ -3664,9 +3682,6 @@
         <v>12</v>
       </c>
       <c r="R70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T70" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3675,62 +3690,156 @@
         <v>0</v>
       </c>
       <c r="B71" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T71" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="72" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B72" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y71" s="2" t="s">
+      <c r="D72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y72" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="73" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y73" s="2" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B999">
+  <conditionalFormatting sqref="A2:B998">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(ISBLANK($C2))</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: generate updated CSV files
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F4B782-8817-4710-9DF4-CF1DC769A440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6D604B-DBE0-43D2-90A1-40228C166814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="98">
   <si>
     <t>FedYYC</t>
   </si>
@@ -327,6 +327,9 @@
   </si>
   <si>
     <t>NewFolder</t>
+  </si>
+  <si>
+    <t>Urban Planning</t>
   </si>
 </sst>
 </file>
@@ -616,7 +619,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1066A4C7-BC62-4C6E-8946-8A1FB62B0DAC}">
-  <dimension ref="A1:AA73"/>
+  <dimension ref="A1:AA74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
@@ -901,6 +904,9 @@
       <c r="K6" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="S6" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -1190,7 +1196,7 @@
         <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>12</v>
@@ -1202,7 +1208,7 @@
         <v>13</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>12</v>
@@ -1211,7 +1217,7 @@
         <v>12</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>13</v>
@@ -1228,157 +1234,139 @@
         <v>0</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V16" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B17" s="1" t="s">
+      <c r="D17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V17" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V17" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z18" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="V18" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D19" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>13</v>
@@ -1386,6 +1374,9 @@
       <c r="J19" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="K19" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="L19" s="2" t="s">
         <v>13</v>
       </c>
@@ -1393,16 +1384,16 @@
         <v>13</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S19" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U19" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W19" s="2" t="s">
         <v>13</v>
@@ -1417,7 +1408,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>0</v>
       </c>
@@ -1425,14 +1416,11 @@
         <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F20" s="2" t="s">
         <v>13</v>
       </c>
@@ -1445,9 +1433,6 @@
       <c r="J20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="L20" s="2" t="s">
         <v>13</v>
       </c>
@@ -1479,7 +1464,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>0</v>
       </c>
@@ -1487,114 +1472,111 @@
         <v>31</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="X21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z21" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z21" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="D22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="S22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="T22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W22" s="2" t="s">
         <v>13</v>
@@ -1609,21 +1591,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>13</v>
@@ -1631,26 +1610,38 @@
       <c r="G23" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="H23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="K23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="R23" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="W23" s="2" t="s">
         <v>13</v>
@@ -1665,7 +1656,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>0</v>
       </c>
@@ -1673,7 +1664,7 @@
         <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>12</v>
@@ -1685,13 +1676,7 @@
         <v>13</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>12</v>
@@ -1699,9 +1684,6 @@
       <c r="L24" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M24" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N24" s="2" t="s">
         <v>12</v>
       </c>
@@ -1730,7 +1712,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>0</v>
       </c>
@@ -1738,7 +1720,7 @@
         <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>12</v>
@@ -1770,9 +1752,6 @@
       <c r="N25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R25" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="S25" s="2" t="s">
         <v>12</v>
       </c>
@@ -1798,7 +1777,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
@@ -1806,7 +1785,7 @@
         <v>91</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>12</v>
@@ -1866,7 +1845,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>0</v>
       </c>
@@ -1874,11 +1853,14 @@
         <v>91</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E27" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="F27" s="2" t="s">
         <v>13</v>
       </c>
@@ -1931,7 +1913,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>0</v>
       </c>
@@ -1939,23 +1921,32 @@
         <v>91</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F28" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M28" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N28" s="2" t="s">
         <v>12</v>
       </c>
@@ -1987,7 +1978,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
@@ -1995,11 +1986,14 @@
         <v>91</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E29" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="F29" s="2" t="s">
         <v>13</v>
       </c>
@@ -2040,7 +2034,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>0</v>
       </c>
@@ -2048,122 +2042,140 @@
         <v>91</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="X30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z30" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z30" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="D31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="X31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z31" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R31" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="D32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA32" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R32" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
@@ -2173,23 +2185,32 @@
       <c r="B33" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="D33" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="S33" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T33" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="Z33" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA33" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
@@ -2200,15 +2221,18 @@
         <v>41</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S34" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T34" s="2" t="s">
@@ -2223,12 +2247,18 @@
         <v>41</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Z35" s="2" t="s">
+      <c r="E35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T35" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2240,12 +2270,12 @@
         <v>41</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="AA36" s="2" t="s">
+      <c r="Z36" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2257,18 +2287,12 @@
         <v>41</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T37" s="2" t="s">
+      <c r="AA37" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2280,12 +2304,18 @@
         <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M38" s="2" t="s">
+      <c r="E38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T38" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2297,12 +2327,12 @@
         <v>41</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H39" s="2" t="s">
+      <c r="M39" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2311,73 +2341,16 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>2</v>
+        <v>41</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y40" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.25">
@@ -2387,14 +2360,71 @@
       <c r="B41" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D41" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y41" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
@@ -2405,73 +2435,13 @@
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F42" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O42" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P42" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X42" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y42" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
@@ -2482,22 +2452,73 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E43" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="F43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="O43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="P43" s="2" t="s">
         <v>12</v>
+      </c>
+      <c r="Q43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y43" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.25">
@@ -2508,12 +2529,15 @@
         <v>2</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O44" s="2" t="s">
@@ -2531,7 +2555,7 @@
         <v>2</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>12</v>
@@ -2554,18 +2578,12 @@
         <v>2</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O46" s="2" t="s">
@@ -2583,7 +2601,7 @@
         <v>2</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>12</v>
@@ -2609,33 +2627,27 @@
         <v>0</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>55</v>
+        <v>2</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K48" s="2" t="s">
+      <c r="F48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V48" s="2" t="s">
+      <c r="O48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P48" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2644,32 +2656,17 @@
         <v>0</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K49" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M49" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N49" s="2" t="s">
         <v>12</v>
       </c>
@@ -2686,15 +2683,6 @@
         <v>12</v>
       </c>
       <c r="V49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X49" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y49" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2703,14 +2691,20 @@
         <v>0</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G50" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H50" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I50" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J50" s="2" t="s">
         <v>12</v>
       </c>
@@ -2727,6 +2721,27 @@
         <v>12</v>
       </c>
       <c r="R50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y50" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2735,58 +2750,31 @@
         <v>0</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y51" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="R51" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
@@ -2796,50 +2784,56 @@
       <c r="B52" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C52" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="S52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V52" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="W52" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X52" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y52" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
@@ -2850,7 +2844,7 @@
         <v>58</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>12</v>
@@ -2892,15 +2886,6 @@
         <v>12</v>
       </c>
       <c r="V53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X53" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y53" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2912,7 +2897,7 @@
         <v>58</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>12</v>
@@ -2954,6 +2939,15 @@
         <v>12</v>
       </c>
       <c r="V54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y54" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2962,11 +2956,20 @@
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H55" s="2" t="s">
         <v>12</v>
       </c>
@@ -2986,9 +2989,6 @@
         <v>12</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R55" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S55" s="2" t="s">
@@ -3009,20 +3009,11 @@
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H56" s="2" t="s">
         <v>12</v>
       </c>
@@ -3057,15 +3048,6 @@
         <v>12</v>
       </c>
       <c r="V56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y56" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3074,17 +3056,26 @@
         <v>0</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G57" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I57" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J57" s="2" t="s">
         <v>12</v>
       </c>
@@ -3113,6 +3104,15 @@
         <v>12</v>
       </c>
       <c r="V57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y57" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3121,11 +3121,14 @@
         <v>0</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G58" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H58" s="2" t="s">
         <v>12</v>
       </c>
@@ -3138,10 +3141,25 @@
       <c r="L58" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R58" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="S58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T58" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="U58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V58" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3150,73 +3168,28 @@
         <v>0</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="R59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y59" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
@@ -3226,20 +3199,71 @@
       <c r="B60" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C60" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S60" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="T60" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="U60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y60" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
@@ -3250,7 +3274,7 @@
         <v>65</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>12</v>
@@ -3258,37 +3282,10 @@
       <c r="G61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S61" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V61" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3300,23 +3297,17 @@
         <v>65</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I62" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3345,9 +3336,6 @@
         <v>12</v>
       </c>
       <c r="V62" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W62" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3359,7 +3347,7 @@
         <v>65</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>12</v>
@@ -3367,9 +3355,6 @@
       <c r="E63" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F63" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3394,15 +3379,6 @@
       <c r="N63" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q63" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3419,12 +3395,6 @@
         <v>12</v>
       </c>
       <c r="W63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y63" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3436,17 +3406,26 @@
         <v>65</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I64" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3462,6 +3441,15 @@
       <c r="N64" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q64" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3475,6 +3463,15 @@
         <v>12</v>
       </c>
       <c r="V64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y64" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3486,7 +3483,7 @@
         <v>65</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>12</v>
@@ -3536,18 +3533,45 @@
         <v>65</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K66" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M66" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="N66" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V66" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3556,36 +3580,21 @@
         <v>0</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L67" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N67" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S67" s="2" t="s">
+      <c r="R67" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3594,12 +3603,21 @@
         <v>0</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G68" s="2" t="s">
+      <c r="F68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J68" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K68" s="2" t="s">
@@ -3611,7 +3629,10 @@
       <c r="M68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R68" s="2" t="s">
+      <c r="N68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S68" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3620,7 +3641,7 @@
         <v>0</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>12</v>
@@ -3628,15 +3649,6 @@
       <c r="G69" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J69" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K69" s="2" t="s">
         <v>12</v>
       </c>
@@ -3646,22 +3658,7 @@
       <c r="M69" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N69" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="R69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V69" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3670,11 +3667,29 @@
         <v>0</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L70" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M70" s="2" t="s">
         <v>12</v>
       </c>
@@ -3682,6 +3697,18 @@
         <v>12</v>
       </c>
       <c r="R70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V70" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3690,20 +3717,11 @@
         <v>0</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K71" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M71" s="2" t="s">
         <v>12</v>
       </c>
@@ -3711,9 +3729,6 @@
         <v>12</v>
       </c>
       <c r="R71" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T71" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3722,29 +3737,20 @@
         <v>0</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="F72" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G72" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J72" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K72" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L72" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M72" s="2" t="s">
         <v>12</v>
       </c>
@@ -3754,25 +3760,7 @@
       <c r="R72" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S72" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X72" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y72" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3781,65 +3769,124 @@
         <v>0</v>
       </c>
       <c r="B73" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y73" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="74" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B74" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y73" s="2" t="s">
+      <c r="D74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y74" s="2" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B998">
+  <conditionalFormatting sqref="A2:B999">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(ISBLANK($C2))</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs - updated permissions
</commit_message>
<xml_diff>
--- a/inputs/file-org-folder-permissions.xlsx
+++ b/inputs/file-org-folder-permissions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrod\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccrodua\Documents\new-file-management-system\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28F8DE1-FBF6-4492-8150-17CDA607B1D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91D45EB-3C12-40FB-A11E-A8C3F53FE1EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
+    <workbookView xWindow="-28920" yWindow="-810" windowWidth="29040" windowHeight="15720" xr2:uid="{E70264EB-E0CC-45A2-B975-12D2A3CA530C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="98">
   <si>
     <t>FedYYC</t>
   </si>
@@ -323,13 +323,13 @@
     <t>Design Desk</t>
   </si>
   <si>
-    <t>PIP</t>
-  </si>
-  <si>
-    <t>NewFolder</t>
-  </si>
-  <si>
-    <t>Urban Planning</t>
+    <t>Organization Culture &amp; EDIB</t>
+  </si>
+  <si>
+    <t>Placemaking Coordinator</t>
+  </si>
+  <si>
+    <t>Urban Planning Intern</t>
   </si>
 </sst>
 </file>
@@ -619,38 +619,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1066A4C7-BC62-4C6E-8946-8A1FB62B0DAC}">
-  <dimension ref="A1:AA74"/>
+  <dimension ref="A1:AC72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="24" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="32.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="17.42578125" style="2" customWidth="1"/>
     <col min="8" max="8" width="19.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="24.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.140625" style="2" customWidth="1"/>
     <col min="10" max="10" width="33" style="2" customWidth="1"/>
     <col min="11" max="11" width="26" style="2" customWidth="1"/>
     <col min="12" max="12" width="25.5703125" style="2" customWidth="1"/>
     <col min="13" max="13" width="13.85546875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="29.28515625" style="2" customWidth="1"/>
-    <col min="15" max="16" width="18" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27" style="2" customWidth="1"/>
-    <col min="19" max="19" width="21.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="51.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="21.140625" style="2" customWidth="1"/>
-    <col min="23" max="23" width="9.140625" style="2"/>
-    <col min="24" max="24" width="15.85546875" style="2" customWidth="1"/>
-    <col min="25" max="25" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="34" style="2" customWidth="1"/>
-    <col min="27" max="27" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="16384" width="9.140625" style="1"/>
+    <col min="14" max="14" width="20.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="29.28515625" style="2" customWidth="1"/>
+    <col min="16" max="17" width="18" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="27" style="2" customWidth="1"/>
+    <col min="20" max="20" width="21.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="51.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="21.140625" style="2" customWidth="1"/>
+    <col min="24" max="24" width="23.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.140625" style="2"/>
+    <col min="26" max="26" width="15.85546875" style="2" customWidth="1"/>
+    <col min="27" max="27" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="34" style="2" customWidth="1"/>
+    <col min="29" max="29" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -691,49 +693,55 @@
         <v>8</v>
       </c>
       <c r="N1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -765,16 +773,16 @@
         <v>13</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U2" s="2" t="s">
         <v>12</v>
@@ -783,7 +791,7 @@
         <v>12</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>13</v>
@@ -794,8 +802,14 @@
       <c r="Z2" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AA2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -814,10 +828,7 @@
       <c r="L3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S3" s="2" t="s">
@@ -832,8 +843,14 @@
       <c r="V3" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="W3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -864,7 +881,7 @@
       <c r="N4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S4" s="2" t="s">
@@ -873,8 +890,14 @@
       <c r="T4" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="U4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -887,11 +910,11 @@
       <c r="K5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="S5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -904,8 +927,11 @@
       <c r="K6" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="U6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -928,7 +954,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>0</v>
       </c>
@@ -947,13 +973,10 @@
       <c r="L8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T8" s="2" t="s">
+      <c r="O8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="U8" s="2" t="s">
@@ -962,8 +985,14 @@
       <c r="V8" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="W8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>0</v>
       </c>
@@ -979,11 +1008,14 @@
       <c r="M9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R9" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="N9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -1017,11 +1049,11 @@
       <c r="M10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N10" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="O10" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -1040,13 +1072,10 @@
       <c r="L11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T11" s="2" t="s">
+      <c r="O11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S11" s="2" t="s">
         <v>12</v>
       </c>
       <c r="U11" s="2" t="s">
@@ -1055,8 +1084,11 @@
       <c r="V11" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="W11" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>0</v>
       </c>
@@ -1090,11 +1122,14 @@
       <c r="N12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R12" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="O12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>0</v>
       </c>
@@ -1129,12 +1164,12 @@
         <v>13</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="W13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="X13" s="2" t="s">
@@ -1143,8 +1178,14 @@
       <c r="Y13" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA13" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
@@ -1181,73 +1222,58 @@
       <c r="M14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="S14" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="N14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="X14" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H15" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I15" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>13</v>
+      <c r="O15" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W15" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>95</v>
+        <v>30</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="H16" s="2" t="s">
         <v>12</v>
       </c>
@@ -1255,87 +1281,141 @@
         <v>12</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X16" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R17" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB17" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="F18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H18" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S18" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="T18" s="2" t="s">
         <v>12</v>
       </c>
@@ -1345,25 +1425,40 @@
       <c r="V18" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB18" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="C19" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="D19" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>13</v>
@@ -1372,7 +1467,7 @@
         <v>13</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>13</v>
@@ -1381,22 +1476,19 @@
         <v>13</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S19" s="2" t="s">
-        <v>27</v>
+        <v>13</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X19" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="V19" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="Y19" s="2" t="s">
         <v>13</v>
@@ -1404,8 +1496,14 @@
       <c r="Z19" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB19" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>0</v>
       </c>
@@ -1413,126 +1511,147 @@
         <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB20" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB21" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z20" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z21" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="D22" s="2" t="s">
         <v>12</v>
       </c>
@@ -1543,13 +1662,7 @@
         <v>13</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>12</v>
@@ -1557,13 +1670,7 @@
       <c r="L22" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S22" s="2" t="s">
+      <c r="O22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T22" s="2" t="s">
@@ -1576,10 +1683,10 @@
         <v>12</v>
       </c>
       <c r="W22" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X22" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y22" s="2" t="s">
         <v>13</v>
@@ -1587,64 +1694,67 @@
       <c r="Z22" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB22" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>91</v>
       </c>
+      <c r="C23" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="D23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="T23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W23" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X23" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y23" s="2" t="s">
         <v>13</v>
@@ -1652,8 +1762,14 @@
       <c r="Z23" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB23" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>0</v>
       </c>
@@ -1661,7 +1777,7 @@
         <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>12</v>
@@ -1673,7 +1789,13 @@
         <v>13</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>12</v>
@@ -1681,9 +1803,15 @@
       <c r="L24" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M24" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N24" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O24" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="S24" s="2" t="s">
         <v>12</v>
       </c>
@@ -1697,10 +1825,10 @@
         <v>12</v>
       </c>
       <c r="W24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y24" s="2" t="s">
         <v>13</v>
@@ -1708,8 +1836,14 @@
       <c r="Z24" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB24" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>0</v>
       </c>
@@ -1717,7 +1851,7 @@
         <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>12</v>
@@ -1749,6 +1883,9 @@
       <c r="N25" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O25" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="S25" s="2" t="s">
         <v>12</v>
       </c>
@@ -1762,10 +1899,10 @@
         <v>12</v>
       </c>
       <c r="W25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y25" s="2" t="s">
         <v>13</v>
@@ -1773,8 +1910,14 @@
       <c r="Z25" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB25" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
@@ -1782,14 +1925,11 @@
         <v>91</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F26" s="2" t="s">
         <v>13</v>
       </c>
@@ -1814,7 +1954,7 @@
       <c r="N26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R26" s="2" t="s">
+      <c r="O26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S26" s="2" t="s">
@@ -1830,10 +1970,10 @@
         <v>12</v>
       </c>
       <c r="W26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y26" s="2" t="s">
         <v>13</v>
@@ -1841,8 +1981,14 @@
       <c r="Z26" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB26" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>0</v>
       </c>
@@ -1850,7 +1996,7 @@
         <v>91</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>12</v>
@@ -1861,28 +2007,13 @@
       <c r="F27" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R27" s="2" t="s">
+      <c r="O27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S27" s="2" t="s">
@@ -1898,10 +2029,10 @@
         <v>12</v>
       </c>
       <c r="W27" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X27" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y27" s="2" t="s">
         <v>13</v>
@@ -1909,8 +2040,14 @@
       <c r="Z27" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB27" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>0</v>
       </c>
@@ -1918,7 +2055,7 @@
         <v>91</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>12</v>
@@ -1926,28 +2063,13 @@
       <c r="F28" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R28" s="2" t="s">
+      <c r="O28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S28" s="2" t="s">
@@ -1963,10 +2085,10 @@
         <v>12</v>
       </c>
       <c r="W28" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X28" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y28" s="2" t="s">
         <v>13</v>
@@ -1974,8 +2096,14 @@
       <c r="Z28" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB28" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
@@ -1983,7 +2111,7 @@
         <v>91</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>12</v>
@@ -1994,19 +2122,16 @@
       <c r="F29" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G29" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K29" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N29" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R29" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S29" s="2" t="s">
+      <c r="O29" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T29" s="2" t="s">
@@ -2019,10 +2144,10 @@
         <v>12</v>
       </c>
       <c r="W29" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X29" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y29" s="2" t="s">
         <v>13</v>
@@ -2030,22 +2155,31 @@
       <c r="Z29" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="AA29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB29" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>13</v>
+      <c r="G30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>12</v>
@@ -2053,99 +2187,66 @@
       <c r="L30" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M30" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R30" s="2" t="s">
+      <c r="O30" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="T30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z30" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="T31" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="U31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V31" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W31" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="X31" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y31" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z31" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="AB31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC31" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>12</v>
@@ -2153,64 +2254,40 @@
       <c r="G32" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K32" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R32" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="T32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U32" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>41</v>
       </c>
+      <c r="C33" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="D33" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S33" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T33" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z33" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA33" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="U33" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>0</v>
       </c>
@@ -2218,25 +2295,16 @@
         <v>41</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T34" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB34" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>0</v>
       </c>
@@ -2244,22 +2312,16 @@
         <v>41</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T35" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AC35" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>0</v>
       </c>
@@ -2267,16 +2329,23 @@
         <v>41</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>44</v>
+        <v>95</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Z36" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="H36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC36" s="2"/>
+    </row>
+    <row r="37" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>0</v>
       </c>
@@ -2284,16 +2353,22 @@
         <v>41</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="AA37" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="E37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U37" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>0</v>
       </c>
@@ -2301,22 +2376,19 @@
         <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T38" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="M38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -2324,107 +2396,113 @@
         <v>41</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M39" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="H39" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA40" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C41" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="D41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X41" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y41" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>0</v>
       </c>
@@ -2432,16 +2510,82 @@
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E42" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="F42" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="43" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="G42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA42" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>0</v>
       </c>
@@ -2449,76 +2593,25 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E43" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O43" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="P43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="Q43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="U43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y43" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44" spans="1:27" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>0</v>
       </c>
@@ -2526,7 +2619,7 @@
         <v>2</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>12</v>
@@ -2534,17 +2627,14 @@
       <c r="F44" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G44" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O44" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="P44" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="45" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Q44" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>0</v>
       </c>
@@ -2552,7 +2642,7 @@
         <v>2</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>12</v>
@@ -2560,14 +2650,14 @@
       <c r="F45" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O45" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="P45" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="46" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Q45" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -2575,7 +2665,7 @@
         <v>2</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>12</v>
@@ -2583,14 +2673,20 @@
       <c r="F46" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O46" s="2" t="s">
+      <c r="G46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="P46" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="47" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Q46" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>0</v>
       </c>
@@ -2598,7 +2694,7 @@
         <v>2</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>12</v>
@@ -2612,30 +2708,24 @@
       <c r="L47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O47" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="P47" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="48" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Q47" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F48" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G48" s="2" t="s">
+      <c r="K48" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L48" s="2" t="s">
@@ -2644,30 +2734,60 @@
       <c r="O48" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P48" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="S48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X48" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="G49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K49" s="2" t="s">
         <v>12</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N49" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R49" s="2" t="s">
+      <c r="O49" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S49" s="2" t="s">
@@ -2682,26 +2802,35 @@
       <c r="V49" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA49" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G50" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H50" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I50" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J50" s="2" t="s">
         <v>12</v>
       </c>
@@ -2714,126 +2843,141 @@
       <c r="M50" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N50" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R50" s="2" t="s">
+      <c r="O50" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S50" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="T50" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="U50" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="V50" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W50" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X50" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y50" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R51" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="O51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z51" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA51" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="52" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>58</v>
       </c>
+      <c r="C52" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="D52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="O52" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="V52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="W52" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="X52" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y52" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="53" spans="1:25" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="53" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>0</v>
       </c>
@@ -2841,7 +2985,7 @@
         <v>58</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>12</v>
@@ -2873,7 +3017,7 @@
       <c r="N53" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S53" s="2" t="s">
+      <c r="O53" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T53" s="2" t="s">
@@ -2885,8 +3029,23 @@
       <c r="V53" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="54" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA53" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>0</v>
       </c>
@@ -2894,7 +3053,7 @@
         <v>58</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>12</v>
@@ -2926,7 +3085,7 @@
       <c r="N54" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S54" s="2" t="s">
+      <c r="O54" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T54" s="2" t="s">
@@ -2944,29 +3103,17 @@
       <c r="X54" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Y54" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="55" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E55" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H55" s="2" t="s">
         <v>12</v>
       </c>
@@ -2988,6 +3135,9 @@
       <c r="N55" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O55" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="S55" s="2" t="s">
         <v>12</v>
       </c>
@@ -3000,17 +3150,29 @@
       <c r="V55" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W55" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="56" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="H56" s="2" t="s">
         <v>12</v>
       </c>
@@ -3032,7 +3194,7 @@
       <c r="N56" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R56" s="2" t="s">
+      <c r="O56" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S56" s="2" t="s">
@@ -3047,32 +3209,38 @@
       <c r="V56" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="57" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA56" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="57" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G57" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I57" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J57" s="2" t="s">
         <v>12</v>
       </c>
@@ -3085,10 +3253,7 @@
       <c r="M57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R57" s="2" t="s">
+      <c r="O57" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S57" s="2" t="s">
@@ -3106,26 +3271,17 @@
       <c r="W57" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="X57" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y57" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G58" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H58" s="2" t="s">
         <v>12</v>
       </c>
@@ -3138,21 +3294,9 @@
       <c r="L58" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M58" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N58" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R58" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="S58" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="T58" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="U58" s="2" t="s">
         <v>12</v>
       </c>
@@ -3160,110 +3304,110 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="M59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="R59" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="S59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T59" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="U59" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="V59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA59" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="60" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>65</v>
       </c>
+      <c r="C60" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="D60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T60" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="V60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="W60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="X60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y60" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="61" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>0</v>
       </c>
@@ -3271,7 +3415,7 @@
         <v>65</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>12</v>
@@ -3279,14 +3423,44 @@
       <c r="G61" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K61" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S61" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="T61" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="62" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="U61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W61" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>0</v>
       </c>
@@ -3294,17 +3468,23 @@
         <v>65</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E62" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I62" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J62" s="2" t="s">
         <v>12</v>
       </c>
@@ -3320,7 +3500,7 @@
       <c r="N62" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R62" s="2" t="s">
+      <c r="O62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S62" s="2" t="s">
@@ -3335,8 +3515,17 @@
       <c r="V62" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="63" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y62" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="63" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>0</v>
       </c>
@@ -3344,7 +3533,7 @@
         <v>65</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>12</v>
@@ -3352,6 +3541,9 @@
       <c r="E63" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="F63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3376,6 +3568,15 @@
       <c r="N63" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="O63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q63" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="R63" s="2" t="s">
         <v>12</v>
       </c>
@@ -3394,8 +3595,20 @@
       <c r="W63" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="X63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA63" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="64" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>0</v>
       </c>
@@ -3403,26 +3616,17 @@
         <v>65</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I64" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3441,15 +3645,6 @@
       <c r="O64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R64" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="S64" s="2" t="s">
         <v>12</v>
       </c>
@@ -3465,14 +3660,8 @@
       <c r="W64" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="X64" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y64" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="65" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>0</v>
       </c>
@@ -3480,7 +3669,7 @@
         <v>65</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>12</v>
@@ -3506,7 +3695,7 @@
       <c r="N65" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R65" s="2" t="s">
+      <c r="O65" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S65" s="2" t="s">
@@ -3521,8 +3710,11 @@
       <c r="V65" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="66" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W65" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="66" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>0</v>
       </c>
@@ -3530,91 +3722,73 @@
         <v>65</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J66" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="K66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L66" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M66" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R66" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="S66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="T66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V66" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="67" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="F67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K67" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L67" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R67" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="68" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="O67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T67" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="68" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I68" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J68" s="2" t="s">
+      <c r="G68" s="2" t="s">
         <v>12</v>
       </c>
       <c r="K68" s="2" t="s">
@@ -3633,12 +3807,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>12</v>
@@ -3646,6 +3820,15 @@
       <c r="G69" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K69" s="2" t="s">
         <v>12</v>
       </c>
@@ -3655,240 +3838,161 @@
       <c r="M69" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R69" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="70" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="N69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X69" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="70" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L70" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="M70" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R70" s="2" t="s">
+      <c r="O70" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="T70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U70" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V70" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="71" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="F71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M71" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N71" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R71" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="72" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="O71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U71" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="72" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F72" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G72" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="K72" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="L72" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="M72" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N72" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R72" s="2" t="s">
+      <c r="O72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S72" s="2" t="s">
         <v>12</v>
       </c>
       <c r="T72" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="73" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X73" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y73" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="74" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X74" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y74" s="2" t="s">
+      <c r="U72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA72" s="2" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B999">
+  <conditionalFormatting sqref="A2:B1000">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(ISBLANK($C2))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:AA1048576">
+  <conditionalFormatting sqref="D1:AC1048576">
     <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>"RW"</formula>
     </cfRule>

</xml_diff>